<commit_message>
DP: create_forecast_basic - current - emp_current_year.ipynb & students_current_year.ipynb - make dynamic
</commit_message>
<xml_diff>
--- a/create_forecast_basic/current/Intermediates/okev_factor.xlsx
+++ b/create_forecast_basic/current/Intermediates/okev_factor.xlsx
@@ -452,10 +452,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.455</v>
+        <v>-2.562</v>
       </c>
       <c r="C2" t="n">
-        <v>0.605</v>
+        <v>-2.412</v>
       </c>
     </row>
     <row r="3">
@@ -465,10 +465,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.305</v>
+        <v>-2.712</v>
       </c>
       <c r="C3" t="n">
-        <v>0.455</v>
+        <v>-2.562</v>
       </c>
     </row>
     <row r="4">
@@ -478,10 +478,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.155</v>
+        <v>-2.862</v>
       </c>
       <c r="C4" t="n">
-        <v>0.305</v>
+        <v>-2.712</v>
       </c>
     </row>
   </sheetData>

</xml_diff>